<commit_message>
Performer: 6.2.4 Alternative Workflow für Fehler in Workflow 6.2.8 erstellt
</commit_message>
<xml_diff>
--- a/Medavis_Performer_Lunatec/Data/Config.xlsx
+++ b/Medavis_Performer_Lunatec/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.jahl\develop\RPA\uipath-rpa_med\Medavis_Performer_Lunatec\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.jahl\develop\uipath\uipath-rpa_med\Medavis_Performer_Lunatec\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81EA64AF-8E74-40C2-9582-82F9E5437684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A39A8E9-9A49-4296-9D47-F4B072A65631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Performer: geprüft und bereit zum Produktivtest
</commit_message>
<xml_diff>
--- a/Medavis_Performer_Lunatec/Data/Config.xlsx
+++ b/Medavis_Performer_Lunatec/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.jahl\develop\uipath\uipath-rpa_med\Medavis_Performer_Lunatec\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A39A8E9-9A49-4296-9D47-F4B072A65631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F33806-79F6-49A5-9F7F-E03DCC9B7D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25605" yWindow="1845" windowWidth="17280" windowHeight="10500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="84">
   <si>
     <t>Name</t>
   </si>
@@ -271,6 +271,12 @@
   </si>
   <si>
     <t>rpa004_InputArchivOrdner</t>
+  </si>
+  <si>
+    <t>rpa004_WebexRoomID</t>
+  </si>
+  <si>
+    <t>rpa004_WebexApiUrl</t>
   </si>
 </sst>
 </file>
@@ -3148,23 +3154,37 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="29" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Performer: in config Prozesse für KillAllProcesses hinzugefügt
</commit_message>
<xml_diff>
--- a/Medavis_Performer_Lunatec/Data/Config.xlsx
+++ b/Medavis_Performer_Lunatec/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.jahl\develop\uipath\uipath-rpa_med\Medavis_Performer_Lunatec\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F33806-79F6-49A5-9F7F-E03DCC9B7D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2992B155-1D5B-45C5-BFA4-C706D9B1B50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25605" yWindow="1845" windowWidth="17280" windowHeight="10500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="85">
   <si>
     <t>Name</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>rpa004_WebexApiUrl</t>
+  </si>
+  <si>
+    <t>ris,excel,outlook</t>
   </si>
 </sst>
 </file>
@@ -1826,6 +1829,9 @@
       <c r="A5" s="5" t="s">
         <v>46</v>
       </c>
+      <c r="B5" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="C5" s="5" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Performer: Prozessnamen für KillAllProcesses schriebweise geändert
</commit_message>
<xml_diff>
--- a/Medavis_Performer_Lunatec/Data/Config.xlsx
+++ b/Medavis_Performer_Lunatec/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.jahl\develop\uipath\uipath-rpa_med\Medavis_Performer_Lunatec\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2992B155-1D5B-45C5-BFA4-C706D9B1B50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE63777-4EA0-4203-AE11-85E6A456B120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -279,7 +279,7 @@
     <t>rpa004_WebexApiUrl</t>
   </si>
   <si>
-    <t>ris,excel,outlook</t>
+    <t>Ris,EXCEL,OUTLOOK</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Performer: Config Werte für Webex Statusmeldung eingetragen; E-Mail WFs gelöscht; Webex WFs Statusmeldung hinzugefügt, Start/Ende/InitException bearbeitet
</commit_message>
<xml_diff>
--- a/Medavis_Performer_Lunatec/Data/Config.xlsx
+++ b/Medavis_Performer_Lunatec/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.jahl\develop\uipath\uipath-rpa_med\Medavis_Performer_Lunatec\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE63777-4EA0-4203-AE11-85E6A456B120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{659F1FC4-0A35-41D7-A041-440DA23D6E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="97">
   <si>
     <t>Name</t>
   </si>
@@ -280,6 +280,42 @@
   </si>
   <si>
     <t>Ris,EXCEL,OUTLOOK</t>
+  </si>
+  <si>
+    <t>CriteriaListSheet</t>
+  </si>
+  <si>
+    <t>EingabeFB_Zusätzliche freieTage</t>
+  </si>
+  <si>
+    <t>CriteriaListDateCell</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>DatabaseFileSheet</t>
+  </si>
+  <si>
+    <t>Datenbank</t>
+  </si>
+  <si>
+    <t>DateColumnName</t>
+  </si>
+  <si>
+    <t>Datum</t>
+  </si>
+  <si>
+    <t>StatusColumnName</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>WebexApiUrl</t>
+  </si>
+  <si>
+    <t>https://webexapis.com/v1/messages</t>
   </si>
 </sst>
 </file>
@@ -747,12 +783,54 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" t="s">
+        <v>96</v>
+      </c>
+    </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>